<commit_message>
Refresh Beijing verified PDFs at 54 keeps (2x schools).
Sync export artifacts after Beijing coverage hit the 2x school target.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/clean/economics/beijing_listings_verified_2026-10-14.xlsx
+++ b/clean/economics/beijing_listings_verified_2026-10-14.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -729,7 +729,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>北京工业大学2026年公开招聘公告（第一批）</t>
+          <t>北京工业大学2026年公开招聘公告（第二批）</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.bjut.edu.cn/info/1072/9076.htm</t>
+          <t>https://www.bjut.edu.cn/info/1072/9464.htm</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -766,37 +766,42 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BJUT</t>
+          <t>Beihang University</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>经济管理学院</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>北京工业大学2026年公开招聘公告（第二批）</t>
+          <t>北京航空航天大学经济管理学院2026年卓越百人博士后岗位招聘通知</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>含师资博士后制度；经管学院岗位见附件</t>
+          <t>含低碳经济、金融工程等方向</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bjut.edu.cn/info/1072/9464.htm</t>
+          <t>http://boshihouzp.gaoxiaozp.com/gxbshzp/57840.html</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>skw@buaa.edu.cn</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -823,12 +828,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>北京航空航天大学经济管理学院2026年卓越百人博士后岗位招聘通知</t>
+          <t>北航经管学院诚邀海内外优秀学者加盟！</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>含低碳经济、金融工程等方向</t>
+          <t>含助理教授及博士后</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -838,7 +843,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>http://boshihouzp.gaoxiaozp.com/gxbshzp/57840.html</t>
+          <t>https://sem.buaa.edu.cn/info/1024/16832.htm</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -848,7 +853,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -865,22 +870,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Beihang University</t>
+          <t>Beijing Normal University</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>经济与工商管理学院</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>北航经管学院诚邀海内外优秀学者加盟！</t>
+          <t>北京师范大学经济与工商管理学院2026年招收博士后公告</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>含助理教授及博士后</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -890,17 +895,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://sem.buaa.edu.cn/info/1024/16832.htm</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>skw@buaa.edu.cn</t>
+          <t>http://boshihoujob.com/gxbsh/beijing/133313.html</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>北京师范大学经济与工商管理学院2026年招收博士后公告</t>
+          <t>北京师范大学经济与工商管理学院2026年招收博士后公告（全球人才网）</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>http://boshihoujob.com/gxbsh/beijing/133313.html</t>
+          <t>https://ifegg.com/html/12654.html</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>北京师范大学经济与工商管理学院2026年招收博士后公告（全球人才网）</t>
+          <t>北京师范大学经济与工商管理学院教学科研岗招聘启事（2026年）</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -989,12 +989,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://ifegg.com/html/12654.html</t>
+          <t>https://bs.bnu.edu.cn/bshzs/e8dc0779c4714d7b937e7a7634f44d20.html</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>bshr@bnu.edu.cn</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1026,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>北京师范大学经济与工商管理学院教学科研岗招聘启事（2026年）</t>
+          <t>北师大经管学院教学科研岗位人才招聘启事（2026年）</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1036,7 +1041,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://bs.bnu.edu.cn/bshzs/e8dc0779c4714d7b937e7a7634f44d20.html</t>
+          <t>https://www.efnchina.com/info/1111/59261.htm</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1063,17 +1068,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Beijing Normal University</t>
+          <t>CAU</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>经济与工商管理学院</t>
+          <t>经济管理学院</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>北师大经管学院教学科研岗位人才招聘启事（2026年）</t>
+          <t>【诚聘】中国农业大学经济管理学院诚聘天下英才</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1088,12 +1093,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.efnchina.com/info/1111/59261.htm</t>
+          <t>https://cem.cau.edu.cn/art/2025/12/16/art_56853_1127416.html</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>bshr@bnu.edu.cn</t>
+          <t>2017062@cau.edu.cn</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1125,27 +1130,22 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>【诚聘】中国农业大学经济管理学院诚聘天下英才</t>
+          <t>中国农业大学2026年度人才招聘启事</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>高层次/普通学术岗全年招聘</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://cem.cau.edu.cn/art/2025/12/16/art_56853_1127416.html</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2017062@cau.edu.cn</t>
+          <t>https://cau.edu.cn/tzgg/7080fc338ac04c4c87c78e37531fef46.htm</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1167,22 +1167,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CAU</t>
+          <t>CUC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>经济与管理学院</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>中国农业大学2026年度人才招聘启事</t>
+          <t>中国传媒大学2026年第二批教学科研岗公开招聘公告</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>高层次/普通学术岗全年招聘</t>
+          <t>含经济与管理学院教学科研岗</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://cau.edu.cn/tzgg/7080fc338ac04c4c87c78e37531fef46.htm</t>
+          <t>https://mkszyxy.cuc.edu.cn/2026/0603/c2346a271304/page.htm</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1214,22 +1214,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CUC</t>
+          <t>CUEB</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>中国传媒大学2026年第二批教学科研岗公开招聘公告</t>
+          <t>首都经济贸易大学2026年公开招聘公告</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>含经济与管理学院教学科研岗</t>
+          <t>教学岗位含经济学院等</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>https://mkszyxy.cuc.edu.cn/2026/0603/c2346a271304/page.htm</t>
+          <t>https://rsj.beijing.gov.cn/xxgk/gkzp/202601/t20260130_4477634.html</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>首都经济贸易大学2026年公开招聘公告</t>
+          <t>首都经济贸易大学2026年公开招聘公告（第二批）</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://rsj.beijing.gov.cn/xxgk/gkzp/202601/t20260130_4477634.html</t>
+          <t>https://rsj.beijing.gov.cn/xxgk/gkzp/202606/t20260630_4740194.html</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1308,22 +1308,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CUEB</t>
+          <t>CUFE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>经济学院/商学院</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>首都经济贸易大学2026年公开招聘公告（第二批）</t>
+          <t>中央财经大学2026年度人才招聘公告（第三批）</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>教学岗位含经济学院等</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://rsj.beijing.gov.cn/xxgk/gkzp/202606/t20260630_4740194.html</t>
+          <t>https://www.cufe.edu.cn/info/1186/26673.htm</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学2026年度人才招聘公告（第三批）</t>
+          <t>中央财经大学2026年度人才招聘公告（第二批）</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>https://www.cufe.edu.cn/info/1186/26673.htm</t>
+          <t>https://www.cufe.edu.cn/info/1186/26420.htm</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学2026年度人才招聘公告（第二批）</t>
+          <t>中央财经大学2026年度教学科研相关岗位人才招聘公告（第一批）</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>含师资博士后通道</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://www.cufe.edu.cn/info/1186/26420.htm</t>
+          <t>https://hr.cufe.edu.cn/info/1046/3431.htm</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>经济学院/商学院</t>
+          <t>应用经济学/理论经济学/工商管理</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学2026年度教学科研相关岗位人才招聘公告（第一批）</t>
+          <t>中央财经大学2026年度第一批博士后研究人员招收简章</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>含师资博士后通道</t>
+          <t>含应用经济学、理论经济学、工商管理流动站</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1474,12 +1474,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>https://hr.cufe.edu.cn/info/1046/3431.htm</t>
+          <t>https://postdoctor.cufe.edu.cn/info/1014/1396.htm</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1506,12 +1506,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学2026年度第一批博士后研究人员招收简章</t>
+          <t>中央财经大学2026年度第一批博士后研究人员招收简章（校官网）</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>含应用经济学、理论经济学、工商管理流动站</t>
+          <t>含应用经济学、理论经济学、工商管理</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>https://postdoctor.cufe.edu.cn/info/1014/1396.htm</t>
+          <t>https://www.cufe.edu.cn/info/1186/26475.htm</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1548,32 +1548,32 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>应用经济学/理论经济学/工商管理</t>
+          <t>商学院</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学2026年度第一批博士后研究人员招收简章（校官网）</t>
+          <t>中央财经大学商学院2026年度教学科研岗招聘公告</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>含应用经济学、理论经济学、工商管理</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>https://www.cufe.edu.cn/info/1186/26475.htm</t>
+          <t>https://bs.cufe.edu.cn/info/1019/10469.htm</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1595,12 +1595,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>商学院</t>
+          <t>商学院、科技商学院</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学商学院2026年度教学科研岗招聘公告</t>
+          <t>中央财经大学商学院、科技商学院2026年度教学科研岗招聘公告（第三批）</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>https://bs.cufe.edu.cn/info/1019/10469.htm</t>
+          <t>http://bs.cufe.edu.cn/info/1019/11089.htm</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1642,12 +1642,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>商学院、科技商学院</t>
+          <t>管理科学与工程学院</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学商学院、科技商学院2026年度教学科研岗招聘公告（第三批）</t>
+          <t>中央财经大学管理科学与工程学院2026年度第一批龙马博士后研究人员招收简章</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>http://bs.cufe.edu.cn/info/1019/11089.htm</t>
+          <t>https://mse.cufe.edu.cn/info/1073/12521.htm</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1689,12 +1689,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>管理科学与工程学院</t>
+          <t>金融学院</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>中央财经大学管理科学与工程学院2026年度第一批龙马博士后研究人员招收简章</t>
+          <t>金融学院2026年度博士后研究人员招收简章</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>https://mse.cufe.edu.cn/info/1073/12521.htm</t>
+          <t>https://sf.cufe.edu.cn/info/1104/15771.htm</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1731,17 +1731,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CUFE</t>
+          <t>CUGB</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>金融学院</t>
+          <t>经济管理学院</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>金融学院2026年度博士后研究人员招收简章</t>
+          <t>中国地质大学（北京）2026年教师岗、实验员岗及专技岗位招聘启事（第二批）</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1751,17 +1751,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>https://sf.cufe.edu.cn/info/1104/15771.htm</t>
+          <t>https://bm.cugb.edu.cn/rscnew/c/2026-04-30/849146.shtml</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CUGB</t>
+          <t>CUP Beijing</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1788,22 +1788,27 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>中国地质大学（北京）2026年教师岗、实验员岗及专技岗位招聘启事（第二批）</t>
+          <t>中国石油大学（北京）经济管理学院诚聘优秀人才</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>全年接受应聘，招满为止</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>https://bm.cugb.edu.cn/rscnew/c/2026-04-30/849146.shtml</t>
+          <t>https://www.cup.edu.cn/sba/rczp/a11fe97eb87141269783d3fded8c4456.htm</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>jgxy@cup.edu.cn</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -1825,42 +1830,37 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CUP Beijing</t>
+          <t>Minzu University</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>中国石油大学（北京）经济管理学院诚聘优秀人才</t>
+          <t>中央民族大学2026年度博士后招收公告</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>全年接受应聘，招满为止</t>
+          <t>普通博士后全年接受申请</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>https://www.cup.edu.cn/sba/rczp/a11fe97eb87141269783d3fded8c4456.htm</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>jgxy@cup.edu.cn</t>
+          <t>https://www.muc.edu.cn/info/1083/49048.htm</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1877,22 +1877,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Minzu University</t>
+          <t>NCEPU</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>经济与管理学院</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>中央民族大学2026年度博士后招收公告</t>
+          <t>华北电力大学2026年度教学科研岗位招聘启事（北京）</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>普通博士后全年接受申请</t>
+          <t>含经济与管理学院教师岗/新讲师博士后</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1902,12 +1902,17 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>https://www.muc.edu.cn/info/1083/49048.htm</t>
+          <t>https://www.ncepu.edu.cn/rczp/bjrczp/e5222acc770e4a7cb8e09eefad9098e1.htm</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>jgxy@ncepu.edu.cn</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1939,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>华北电力大学2026年度教学科研岗位招聘启事（北京）</t>
+          <t>华北电力大学2026年度教学科研岗位招聘启事（含应用经济学）</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>含经济与管理学院教师岗/新讲师博士后</t>
+          <t>含应用经济学等</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1949,7 +1954,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>https://www.ncepu.edu.cn/rczp/bjrczp/e5222acc770e4a7cb8e09eefad9098e1.htm</t>
+          <t>https://www.ncepu.edu.cn/rczp/bdrczp/c9e86b816a9e4c359d3bd2695f737a3a.htm</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1976,37 +1981,37 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NCEPU</t>
+          <t>Peking University</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>光华管理学院</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>华北电力大学2026年度教学科研岗位招聘启事（含应用经济学）</t>
+          <t>2025年北京大学光华管理学院教学科研岗位招聘启事</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>含应用经济学等</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>https://www.ncepu.edu.cn/rczp/bdrczp/c9e86b816a9e4c359d3bd2695f737a3a.htm</t>
+          <t>https://hr.pku.edu.cn/rczp/jxky/a92f835c47714f1ababadf98678a5085.htm</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>jgxy@ncepu.edu.cn</t>
+          <t>recruitment@gsm.pku.edu.cn</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2033,12 +2038,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>光华管理学院</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026年北京大学光华管理学院教学科研岗位招聘启事</t>
+          <t>2025年北京大学经济学院教学科研岗位招聘启事</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2053,12 +2058,12 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>https://hr.pku.edu.cn/rczp/jxky/5a8411beae2c4e8ba518ba4c6efe8794.htm</t>
+          <t>https://hr.pku.edu.cn/rczp/jxky/f5471d5b1df745db9ff270ba2f4fc7db.htm</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>recruitment@gsm.pku.edu.cn</t>
+          <t>econ_pku_hr@163.com</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2085,12 +2090,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>光华管理学院</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026年北京大学经济学院教学科研岗位招聘启事</t>
+          <t>2026年北京大学光华管理学院教学科研岗位招聘启事</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2105,12 +2110,12 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>https://hr.pku.edu.cn/rczp/jxky/aba345dfa9d040df8b64488f3af5b37a.htm</t>
+          <t>https://hr.pku.edu.cn/rczp/jxky/5a8411beae2c4e8ba518ba4c6efe8794.htm</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>econ_pku_hr@163.com</t>
+          <t>recruitment@gsm.pku.edu.cn</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2142,7 +2147,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>北京大学经济学院2026年教职招聘通知</t>
+          <t>2026年北京大学经济学院教学科研岗位招聘启事</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2157,7 +2162,12 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>https://econ.pku.edu.cn/tzgg/50170econ391389.htm</t>
+          <t>https://hr.pku.edu.cn/rczp/jxky/aba345dfa9d040df8b64488f3af5b37a.htm</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>econ_pku_hr@163.com</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2189,12 +2199,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>北京大学经济学院“奥园博士后”项目申请公告</t>
+          <t>北京大学经济学院2026年教职招聘通知</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>全年滚动招收</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2204,12 +2214,12 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>https://econ.pku.edu.cn/tzgg/50170econ372315.htm</t>
+          <t>https://econ.pku.edu.cn/tzgg/50170econ391389.htm</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2246,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>北京大学经济学院面向海内外诚聘英才</t>
+          <t>北京大学经济学院“奥园博士后”项目申请公告</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>全年滚动招收</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2251,17 +2261,12 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>https://econ.pku.edu.cn/tzgg/334008.htm</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>econ_pku_hr@163.com</t>
+          <t>https://econ.pku.edu.cn/tzgg/50170econ372315.htm</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -2278,22 +2283,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Renmin University of China</t>
+          <t>Peking University</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>商学院</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>中国人民大学商学院年度教师招聘（滚动至2026-12-31）</t>
+          <t>北京大学经济学院面向海内外诚聘英才</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>滚动招聘，招满即止</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2303,12 +2308,12 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>https://www.rmbs.ruc.edu.cn/szyky/rczp/ndjszp/97756c032dac49fab16e5a273f0ebf9d.htm</t>
+          <t>https://econ.pku.edu.cn/tzgg/334008.htm</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>recruitment@rmbs.ruc.edu.cn</t>
+          <t>econ_pku_hr@163.com</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2335,17 +2340,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>应用经济学院</t>
+          <t>商学院</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>中国人民大学应用经济学院博士后招聘公告</t>
+          <t>中国人民大学商学院年度教师招聘（滚动至2026-12-31）</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>滚动招聘，招满即止</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2355,12 +2360,17 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>http://ae.ruc.edu.cn/xwzx/tzgg/62a1d3280023497a9cc7a2c15c5894c7.htm</t>
+          <t>https://www.rmbs.ruc.edu.cn/szyky/rczp/ndjszp/97756c032dac49fab16e5a273f0ebf9d.htm</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>recruitment@rmbs.ruc.edu.cn</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -2382,17 +2392,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>财政金融学院</t>
+          <t>应用经济学院</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>中国人民大学财政金融学院2026年度引进人才和教师通知</t>
+          <t>中国人民大学应用经济学院博士后招聘公告</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>滚动招聘，招满即止</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2402,12 +2412,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>https://ifegg.com/html/11188.html</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>cjzonghe@ruc.edu.cn</t>
+          <t>http://ae.ruc.edu.cn/xwzx/tzgg/62a1d3280023497a9cc7a2c15c5894c7.htm</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2434,32 +2439,37 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>财政金融学院/经济学院</t>
+          <t>财政金融学院</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>独树一帜走新路 汇聚英才谱新篇——关于中国人民大学2026年度人才引进和教师招聘通知</t>
+          <t>中国人民大学财政金融学院2026年度引进人才和教师通知</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>含财政金融学院、经济学院等</t>
+          <t>滚动招聘，招满即止</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>http://hr.ruc.edu.cn/zpxx/c26637043fc8457496f0781066bcad04.htm</t>
+          <t>https://ifegg.com/html/11188.html</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>cjzonghe@ruc.edu.cn</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -2481,32 +2491,27 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>财政金融学院</t>
+          <t>财政金融学院/经济学院</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>财政金融学院2026年度人才引进和教师招聘通知</t>
+          <t>独树一帜走新路 汇聚英才谱新篇——关于中国人民大学2026年度人才引进和教师招聘通知</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>滚动招聘，招满即止</t>
+          <t>含财政金融学院、经济学院等</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>http://sf.ruc.edu.cn/sylm/gg_sy/gg/67fefa2748ef4125aa908c2f3bfed087.htm</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>cjzonghe@ruc.edu.cn</t>
+          <t>http://hr.ruc.edu.cn/zpxx/c26637043fc8457496f0781066bcad04.htm</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -2528,22 +2533,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
+          <t>Renmin University of China</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>财政金融学院</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>清华大学经济管理学院2026年招聘教研系列教师（经济系）</t>
+          <t>财政金融学院2026年度人才引进和教师招聘通知</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>截止日期2026-12-31</t>
+          <t>滚动招聘，招满即止</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2553,12 +2558,17 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>https://www.gaoxiaojob.com/announcement/detail/381907.html</t>
+          <t>http://sf.ruc.edu.cn/sylm/gg_sy/gg/67fefa2748ef4125aa908c2f3bfed087.htm</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>cjzonghe@ruc.edu.cn</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2595,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>清华大学经济管理学院应用经济学流动站（合作导师董丰）2026年招聘博士后</t>
+          <t>清华大学经济管理学院2026年招聘教研系列教师（经济系）</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2600,12 +2610,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>https://www.gaoxiaojob.com/announcement/detail/395746.html</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>postdoc@sem.tsinghua.edu.cn</t>
+          <t>https://www.gaoxiaojob.com/announcement/detail/381907.html</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -2637,12 +2642,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>清华大学经济管理学院教师招聘（2026年10月更新）</t>
+          <t>清华大学经济管理学院博士后招聘</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>常年招聘</t>
+          <t>招满即止</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2652,17 +2657,17 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>https://www.sem.tsinghua.edu.cn/js/jszp.htm</t>
+          <t>https://sem.tsinghua.edu.cn/js/bshldz/bshzp.htm</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>scholar@sem.tsinghua.edu.cn</t>
+          <t>postdoc@sem.tsinghua.edu.cn</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -2679,22 +2684,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>UIBE</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>中国金融学院</t>
+          <t>经济管理学院</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>中国金融学院2026年专职教师招聘公告</t>
+          <t>清华大学经济管理学院应用经济学流动站（合作导师董丰）2026年招聘博士后</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>See announcement page</t>
+          <t>截止日期2026-12-31</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2704,12 +2709,17 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>https://sbf.uibe.edu.cn/tzgg/b20abafc23f940349876baa87054aace.htm</t>
+          <t>https://www.gaoxiaojob.com/announcement/detail/395746.html</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>postdoc@sem.tsinghua.edu.cn</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -2726,37 +2736,42 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>UIBE</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>国际经济贸易学院</t>
+          <t>经济管理学院</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>对外经济贸易大学2026年度事业编专职教学科研人员、师资博士后招聘公告</t>
+          <t>清华大学经济管理学院教师招聘（2026年10月更新）</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>含国际经济贸易学院等经管岗位</t>
+          <t>常年招聘</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>https://hr.uibe.edu.cn/jszp/zpxx/654c850954d7459abbde78b5ebc62820.htm</t>
+          <t>https://www.sem.tsinghua.edu.cn/js/jszp.htm</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>scholar@sem.tsinghua.edu.cn</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2793,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>国际经济贸易学院/中国金融学院/经济学院</t>
+          <t>中国金融学院</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>对外经济贸易大学全球价值链研究院专职教学科研人员招聘相关公告</t>
+          <t>中国金融学院2026年专职教师招聘公告</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2793,12 +2808,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Dept/HR</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>https://hr.uibe.edu.cn/jszp/zpxx/ed338932d6d94149945898e2ab2429c7.htm</t>
+          <t>https://sbf.uibe.edu.cn/tzgg/b20abafc23f940349876baa87054aace.htm</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -2825,32 +2840,32 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>全球创新与治理研究院</t>
+          <t>国际经济贸易学院</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>对外经济贸易大学全球创新与治理研究院2025年专职教学科研人员招聘公告</t>
+          <t>对外经济贸易大学2026年度事业编专职教学科研人员、师资博士后招聘公告</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>产业经济学方向</t>
+          <t>含国际经济贸易学院等经管岗位</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>https://agig.uibe.edu.cn/tzgg/e30c29f3c079417eadaaedb5f16dfc54.htm</t>
+          <t>https://hr.uibe.edu.cn/jszp/zpxx/654c850954d7459abbde78b5ebc62820.htm</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -2867,37 +2882,32 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>USTB</t>
+          <t>UIBE</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>国际经济贸易学院/中国金融学院/经济学院</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>经济管理学院2025年诚聘海内外英才</t>
+          <t>对外经济贸易大学全球价值链研究院专职教学科研人员招聘相关公告</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>常年招聘教师/博士后</t>
+          <t>See announcement page</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Dept/HR</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>https://sem.ustb.edu.cn/xwzx/tzgg/a2ffc3d9c3d9495baeba6c87e507644c.htm</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>jgzp@ustb.edu.cn</t>
+          <t>https://hr.uibe.edu.cn/jszp/zpxx/ed338932d6d94149945898e2ab2429c7.htm</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -2919,22 +2929,22 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>USTB</t>
+          <t>UIBE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>经济管理学院</t>
+          <t>全球创新与治理研究院</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>经济管理学院2025年诚聘海内外英才（人才招聘栏目）</t>
+          <t>对外经济贸易大学全球创新与治理研究院2025年专职教学科研人员招聘公告</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>常年招聘</t>
+          <t>产业经济学方向</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2944,12 +2954,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>https://sem.ustb.edu.cn/rczp/a2ffc3d9c3d9495baeba6c87e507644c.htm</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>jgzp@ustb.edu.cn</t>
+          <t>https://agig.uibe.edu.cn/tzgg/e30c29f3c079417eadaaedb5f16dfc54.htm</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -2981,30 +2986,186 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
+          <t>北京科技大学经济管理学院博士后招聘</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>含经济学、金融学等领域</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.ustb.edu.cn/szll/bshldz/bshzp/index.htm</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>jgzp@ustb.edu.cn</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>USTB</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>经济管理学院2025年诚聘海内外英才</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>常年招聘教师/博士后</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.ustb.edu.cn/xwzx/tzgg/a2ffc3d9c3d9495baeba6c87e507644c.htm</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>jgzp@ustb.edu.cn</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>USTB</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>经济管理学院2025年诚聘海内外英才（人才招聘栏目）</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>常年招聘</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.ustb.edu.cn/rczp/a2ffc3d9c3d9495baeba6c87e507644c.htm</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>jgzp@ustb.edu.cn</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>USTB</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>经济管理学院</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
           <t>经济管理学院诚聘海内外英才（师资队伍招聘页）</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>常年招聘</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Dept/HR</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>https://sem.ustb.edu.cn/szll/jszp/index.htm</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>jgzp@ustb.edu.cn</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>Academic</t>
         </is>
@@ -3114,6 +3275,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>